<commit_message>
Ajout du test de biais proportionnel Bland-Altman
</commit_message>
<xml_diff>
--- a/data/final/validity_results_all.xlsx
+++ b/data/final/validity_results_all.xlsx
@@ -353,7 +353,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N3"/>
+  <dimension ref="A1:P3"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -427,6 +427,16 @@
           <t>LoA_upper</t>
         </is>
       </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>BA_slope</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>BA_slope_p</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -473,6 +483,12 @@
       <c r="N2">
         <v>87.13213895518319</v>
       </c>
+      <c r="O2">
+        <v>0.2540754335369597</v>
+      </c>
+      <c r="P2">
+        <v>1.478740053326337E-10</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -518,6 +534,12 @@
       </c>
       <c r="N3">
         <v>-6.483318197415642</v>
+      </c>
+      <c r="O3">
+        <v>-0.6626040291396081</v>
+      </c>
+      <c r="P3">
+        <v>6.40312732578966E-31</v>
       </c>
     </row>
   </sheetData>
@@ -527,7 +549,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N4"/>
+  <dimension ref="A1:P4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -601,6 +623,16 @@
           <t>LoA_upper</t>
         </is>
       </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>BA_slope</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>BA_slope_p</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -647,6 +679,12 @@
       <c r="N2">
         <v>1724.868786502032</v>
       </c>
+      <c r="O2">
+        <v>1.097961214607456</v>
+      </c>
+      <c r="P2">
+        <v>1.02515645142164E-27</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -693,6 +731,12 @@
       <c r="N3">
         <v>1299.876214717267</v>
       </c>
+      <c r="O3">
+        <v>0.5671736437324914</v>
+      </c>
+      <c r="P3">
+        <v>4.021153234102253E-14</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -738,6 +782,12 @@
       </c>
       <c r="N4">
         <v>1548.031194279133</v>
+      </c>
+      <c r="O4">
+        <v>0.7692751327749411</v>
+      </c>
+      <c r="P4">
+        <v>3.572251522094927E-16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
changement de qom tete car marqueur mauvais
</commit_message>
<xml_diff>
--- a/data/final/validity_results_all.xlsx
+++ b/data/final/validity_results_all.xlsx
@@ -448,46 +448,46 @@
         <v>120</v>
       </c>
       <c r="C2">
-        <v>0.9234101115287354</v>
+        <v>0.9234101115287343</v>
       </c>
       <c r="D2">
-        <v>0.8917682464640166</v>
+        <v>0.8917682464640151</v>
       </c>
       <c r="E2">
-        <v>0.9460651232431769</v>
+        <v>0.9460651232431762</v>
       </c>
       <c r="F2">
-        <v>6.689872626229933E-51</v>
+        <v>6.689872626235456E-51</v>
       </c>
       <c r="G2">
-        <v>0.8526862340735116</v>
+        <v>0.8526862340735095</v>
       </c>
       <c r="H2">
-        <v>0.8421603242505259</v>
+        <v>0.8421594323834386</v>
       </c>
       <c r="I2">
-        <v>0.5202858641317637</v>
+        <v>0.5202782558418642</v>
       </c>
       <c r="J2">
-        <v>0.9288352378944715</v>
+        <v>0.9288352161356226</v>
       </c>
       <c r="K2">
-        <v>40.28367145604221</v>
+        <v>40.2836714560441</v>
       </c>
       <c r="L2">
-        <v>25.06961702256125</v>
+        <v>25.06961702256327</v>
       </c>
       <c r="M2">
-        <v>-36.99290491006071</v>
+        <v>-36.99290491006023</v>
       </c>
       <c r="N2">
-        <v>87.13213895518319</v>
+        <v>87.13213895518678</v>
       </c>
       <c r="O2">
-        <v>0.2540754335369597</v>
+        <v>0.2540754335369901</v>
       </c>
       <c r="P2">
-        <v>1.478740053326337E-10</v>
+        <v>1.478740053320287E-10</v>
       </c>
     </row>
     <row r="3">
@@ -500,46 +500,46 @@
         <v>120</v>
       </c>
       <c r="C3">
-        <v>0.8788008425067078</v>
+        <v>0.8257433869993704</v>
       </c>
       <c r="D3">
-        <v>0.8303548779173361</v>
+        <v>0.7588117670250647</v>
       </c>
       <c r="E3">
-        <v>0.9140615469034061</v>
+        <v>0.8754166301377868</v>
       </c>
       <c r="F3">
-        <v>1.01290386508408E-39</v>
+        <v>3.996430560945545E-31</v>
       </c>
       <c r="G3">
-        <v>0.7722909207904993</v>
+        <v>0.681852141173192</v>
       </c>
       <c r="H3">
-        <v>0.2598665410598678</v>
+        <v>0.8221427192577244</v>
       </c>
       <c r="I3">
-        <v>-0.06242129397358923</v>
+        <v>0.7541126707309673</v>
       </c>
       <c r="J3">
-        <v>0.6097641350755771</v>
+        <v>0.872684309057678</v>
       </c>
       <c r="K3">
-        <v>30.92786156283232</v>
+        <v>5.814805148316804</v>
       </c>
       <c r="L3">
-        <v>-28.77873304890491</v>
+        <v>-0.9106382282781132</v>
       </c>
       <c r="M3">
-        <v>-51.07414790039419</v>
+        <v>-12.21422560529622</v>
       </c>
       <c r="N3">
-        <v>-6.483318197415642</v>
+        <v>10.39294914874</v>
       </c>
       <c r="O3">
-        <v>-0.6626040291396081</v>
+        <v>0.05921723355329524</v>
       </c>
       <c r="P3">
-        <v>6.40312732578966E-31</v>
+        <v>0.2995813249308721</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
modifie readme et code
</commit_message>
<xml_diff>
--- a/data/final/validity_results_all.xlsx
+++ b/data/final/validity_results_all.xlsx
@@ -862,7 +862,7 @@
         <v>120</v>
       </c>
       <c r="C2">
-        <v>0.6610114287165626</v>
+        <v>0.7674877758252703</v>
       </c>
       <c r="D2">
         <v>0.3137309598237173</v>
@@ -874,7 +874,7 @@
         <v>16.91250523511112</v>
       </c>
       <c r="G2">
-        <v>0.6884104964641545</v>
+        <v>0.8083568000255449</v>
       </c>
       <c r="H2">
         <v>0.3096164958192597</v>
@@ -896,7 +896,7 @@
         <v>120</v>
       </c>
       <c r="C3">
-        <v>0.6785363375710531</v>
+        <v>0.8038957420778015</v>
       </c>
       <c r="D3">
         <v>0.3372523805354467</v>
@@ -908,7 +908,7 @@
         <v>21.82297916845243</v>
       </c>
       <c r="G3">
-        <v>0.6884104964641545</v>
+        <v>0.8083568000255449</v>
       </c>
       <c r="H3">
         <v>0.3096164958192597</v>
@@ -930,7 +930,7 @@
         <v>120</v>
       </c>
       <c r="C4">
-        <v>0.1187706503569854</v>
+        <v>0.1420663889443681</v>
       </c>
       <c r="D4">
         <v>0.3915910931802877</v>
@@ -942,7 +942,7 @@
         <v>27.93864672198165</v>
       </c>
       <c r="G4">
-        <v>0.6884104964641545</v>
+        <v>0.8083568000255449</v>
       </c>
       <c r="H4">
         <v>0.3096164958192597</v>

</xml_diff>